<commit_message>
Correct five errors in Measures of Central Tendency
The headline U.S. CPI is a weighted price index; the trimmed-mean CPI is
the Cleveland Fed's separate gauge. The salary roster has no executive
level, so the skew comes from senior and lead salaries. Job level is
ordered, so it has a median as well as a mode (Mid for both). The
notebook's outlier line printed 'up by hundreds' and 'moved by $1k' for
shifts of 119k and 0.5k, and now computes them, and the solutions'
grouped mean is 28.0 seconds, as the cell prints. The workbook's Notes
sheet says the same.
</commit_message>
<xml_diff>
--- a/data/measures-of-central-tendency--salaries.xlsx
+++ b/data/measures-of-central-tendency--salaries.xlsx
@@ -5652,14 +5652,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>annual_salary is right-skewed: a handful of senior/executive salaries pull the mean above the median, the chapter's core lesson.</t>
+          <t>annual_salary is right-skewed: a handful of senior and lead salaries pull the mean above the median, the chapter's core lesson.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>department and job_level are categorical, so their typical value is a mode, not a mean.</t>
+          <t>department is an unordered category, so its typical value is a mode. job_level is ordered, so it has a median as well.</t>
         </is>
       </c>
     </row>

</xml_diff>